<commit_message>
Update college dashboard application and backend loader/app
</commit_message>
<xml_diff>
--- a/colleges.xlsx
+++ b/colleges.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fe091929957c81be/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fe091929957c81be/Desktop/college Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="774" documentId="13_ncr:1_{3EB9814A-FE3D-40BC-9A46-1A8C0E484E7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5DF5A21-5BDF-430E-8233-4C87D8A83AD7}"/>
+  <xr:revisionPtr revIDLastSave="778" documentId="13_ncr:1_{3EB9814A-FE3D-40BC-9A46-1A8C0E484E7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F5B22B5-4DDB-495C-97CF-06DC41749546}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{E51DEF15-1794-4A01-8E1F-673800EDB52A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E51DEF15-1794-4A01-8E1F-673800EDB52A}"/>
   </bookViews>
   <sheets>
     <sheet name="colleges" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2126" uniqueCount="1052">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2126" uniqueCount="1054">
   <si>
     <t>college_id</t>
   </si>
@@ -3187,6 +3187,12 @@
   </si>
   <si>
     <t>Dr. George Abraham</t>
+  </si>
+  <si>
+    <t>https://cknc.edu.in/</t>
+  </si>
+  <si>
+    <t>https://qmgcw.edu.in/</t>
   </si>
 </sst>
 </file>
@@ -3679,11 +3685,10 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -3741,10 +3746,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4329,8 +4330,8 @@
       <c r="D9" t="s">
         <v>13</v>
       </c>
-      <c r="F9" t="s">
-        <v>43</v>
+      <c r="F9" s="2" t="s">
+        <v>1052</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>656</v>
@@ -4841,8 +4842,8 @@
       <c r="D25" t="s">
         <v>13</v>
       </c>
-      <c r="F25" t="s">
-        <v>43</v>
+      <c r="F25" s="2" t="s">
+        <v>1053</v>
       </c>
       <c r="G25" t="s">
         <v>681</v>
@@ -5847,10 +5848,10 @@
       <c r="I57" t="s">
         <v>102</v>
       </c>
-      <c r="J57" s="3" t="s">
+      <c r="J57" t="s">
         <v>740</v>
       </c>
-      <c r="K57" s="3" t="s">
+      <c r="K57" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5943,7 +5944,7 @@
       <c r="I60" t="s">
         <v>102</v>
       </c>
-      <c r="J60" s="3" t="s">
+      <c r="J60" t="s">
         <v>745</v>
       </c>
       <c r="K60" t="s">
@@ -5975,10 +5976,10 @@
       <c r="I61" t="s">
         <v>78</v>
       </c>
-      <c r="J61" s="3" t="s">
+      <c r="J61" t="s">
         <v>746</v>
       </c>
-      <c r="K61" s="3" t="s">
+      <c r="K61" t="s">
         <v>22</v>
       </c>
     </row>
@@ -6097,10 +6098,10 @@
       <c r="G65" t="s">
         <v>763</v>
       </c>
-      <c r="H65" s="3" t="s">
+      <c r="H65" t="s">
         <v>764</v>
       </c>
-      <c r="I65" s="3" t="s">
+      <c r="I65" t="s">
         <v>56</v>
       </c>
       <c r="J65" t="s">
@@ -6132,7 +6133,7 @@
       <c r="H66" t="s">
         <v>768</v>
       </c>
-      <c r="I66" s="3" t="s">
+      <c r="I66" t="s">
         <v>56</v>
       </c>
       <c r="J66" t="s">
@@ -6164,7 +6165,7 @@
       <c r="H67">
         <v>9444405816</v>
       </c>
-      <c r="I67" s="3" t="s">
+      <c r="I67" t="s">
         <v>112</v>
       </c>
       <c r="J67" t="s">
@@ -10131,7 +10132,7 @@
       <c r="D192" t="s">
         <v>13</v>
       </c>
-      <c r="F192" t="s">
+      <c r="F192" s="2" t="s">
         <v>526</v>
       </c>
       <c r="G192" t="s">
@@ -10323,7 +10324,7 @@
       <c r="D198" t="s">
         <v>13</v>
       </c>
-      <c r="F198" t="s">
+      <c r="F198" s="2" t="s">
         <v>529</v>
       </c>
       <c r="G198" t="s">
@@ -11910,8 +11911,12 @@
     <hyperlink ref="G159" r:id="rId27" xr:uid="{304715CB-4D6A-4801-8BB9-A5A047367C38}"/>
     <hyperlink ref="G208" r:id="rId28" xr:uid="{B98DD5AC-AAFF-4A78-B850-8FEBF92DE6F2}"/>
     <hyperlink ref="G246" r:id="rId29" xr:uid="{81BBCBE3-54B5-4E9D-AD59-2F33D8D2B688}"/>
+    <hyperlink ref="F9" r:id="rId30" xr:uid="{BCE22CB7-D7A1-4047-9005-C18FC1B67E48}"/>
+    <hyperlink ref="F25" r:id="rId31" xr:uid="{C2015A5C-A316-40C1-BBDD-E712AA5D56F7}"/>
+    <hyperlink ref="F198" r:id="rId32" xr:uid="{D6E2F6AE-E0BC-49FC-9FDE-BE3269EFD2CA}"/>
+    <hyperlink ref="F192" r:id="rId33" xr:uid="{F7A220F9-A067-4A49-806D-4CA257A5A992}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId30"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId34"/>
 </worksheet>
 </file>
</xml_diff>